<commit_message>
Add CustomTkinter GUI and clean folder structure (v2)
</commit_message>
<xml_diff>
--- a/output/10_AAM.xlsx
+++ b/output/10_AAM.xlsx
@@ -441,8 +441,10 @@
           <t>EPF</t>
         </is>
       </c>
-      <c r="B2" s="13" t="n">
-        <v>10</v>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="10">
@@ -534,7 +536,7 @@
         </is>
       </c>
       <c r="B14" s="15" t="n">
-        <v>0</v>
+        <v>1833.025</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="10">
@@ -543,8 +545,9 @@
           <t>Total for EPF</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n">
-        <v>20000</v>
+      <c r="B15" s="17">
+        <f>SUM(B10:B14)</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="10">
@@ -554,7 +557,7 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="10">
@@ -614,7 +617,7 @@
         </is>
       </c>
       <c r="B23" s="15" t="n">
-        <v>0</v>
+        <v>1833.025</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="10">
@@ -624,7 +627,7 @@
         </is>
       </c>
       <c r="B24" s="15" t="n">
-        <v>0</v>
+        <v>9080</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="10">
@@ -634,7 +637,7 @@
         </is>
       </c>
       <c r="B25" s="15" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="10">
@@ -674,7 +677,7 @@
         </is>
       </c>
       <c r="B29" s="15" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="10">
@@ -704,7 +707,7 @@
         </is>
       </c>
       <c r="B32" s="15" t="n">
-        <v>0</v>
+        <v>6592</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="10">
@@ -724,7 +727,7 @@
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>0</v>
+        <v>17406.73</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="10">
@@ -733,8 +736,9 @@
           <t>Gross Salary</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n">
-        <v>85000</v>
+      <c r="B35" s="18">
+        <f>B15+SUM(B17:B34)</f>
+        <v/>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="10">
@@ -750,8 +754,9 @@
           <t>EPF 8%</t>
         </is>
       </c>
-      <c r="B38" s="15" t="n">
-        <v>1600</v>
+      <c r="B38" s="15">
+        <f>B15*0.08</f>
+        <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="10">
@@ -771,7 +776,7 @@
         </is>
       </c>
       <c r="B40" s="15" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="10">
@@ -801,7 +806,7 @@
         </is>
       </c>
       <c r="B43" s="15" t="n">
-        <v>0</v>
+        <v>341.8439716312057</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="10">
@@ -831,7 +836,7 @@
         </is>
       </c>
       <c r="B46" s="15" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="10">
@@ -851,7 +856,7 @@
         </is>
       </c>
       <c r="B48" s="15" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="10">
@@ -860,8 +865,9 @@
           <t>Total Deductions</t>
         </is>
       </c>
-      <c r="B49" s="17" t="n">
-        <v>16679.5</v>
+      <c r="B49" s="17">
+        <f>SUM(B38:B48)</f>
+        <v/>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="10">
@@ -870,8 +876,9 @@
           <t>Net Salary</t>
         </is>
       </c>
-      <c r="B50" s="17" t="n">
-        <v>68320.5</v>
+      <c r="B50" s="17">
+        <f>B35-B49</f>
+        <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="10">
@@ -891,8 +898,9 @@
           <t>EPF 12%</t>
         </is>
       </c>
-      <c r="B53" s="15" t="n">
-        <v>7833.599999999999</v>
+      <c r="B53" s="15">
+        <f>B15*0.12</f>
+        <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="10">
@@ -901,8 +909,9 @@
           <t>ETF 3%</t>
         </is>
       </c>
-      <c r="B54" s="15" t="n">
-        <v>1958.4</v>
+      <c r="B54" s="15">
+        <f>B15*0.03</f>
+        <v/>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="10">
@@ -922,7 +931,7 @@
         </is>
       </c>
       <c r="B56" s="15" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="10">
@@ -932,7 +941,7 @@
         </is>
       </c>
       <c r="B57" s="15" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>